<commit_message>
feat: update training log Excel file with new data
</commit_message>
<xml_diff>
--- a/模型比較表格.xlsx
+++ b/模型比較表格.xlsx
@@ -1,31 +1,42 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\barry\Documents\barry-cs-project\ReStraV\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\barry univ 3 fall\資訊工程專題\MyReStraV\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C2F7B9C3-5373-41AB-A218-FEF86B07F2B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8534B19-44E8-434D-9BA8-42C33437512C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{05AB7D64-A468-42E7-95FA-F2D5B1FDA5E0}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{05AB7D64-A468-42E7-95FA-F2D5B1FDA5E0}"/>
   </bookViews>
   <sheets>
     <sheet name="工作表1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="25">
   <si>
     <t>Pika</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -91,10 +102,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>Samples(two_h5_future_set)</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>Sora</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -104,6 +111,30 @@
   </si>
   <si>
     <t>Samples(two_h5_future_set_31_dim)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Samples(two_h5_future_set_22_dim)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Samples(two_h5_future_set_17_dim)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Samples(two_h5_future_set_8_dim)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>REAL</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Samples(two_h5_future_set_21dim(original))</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Samples(two_h5_future_set_13_dim)</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -175,9 +206,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 佈景主題">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 主題">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -215,7 +246,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -321,7 +352,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -463,7 +494,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -471,16 +502,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DB844DEF-FE45-489B-B4F7-DB0202A7BB22}">
-  <dimension ref="A1:T62"/>
-  <sheetFormatPr defaultRowHeight="16.2" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:AV62"/>
+  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="15.109375" customWidth="1"/>
-    <col min="8" max="8" width="20.109375" customWidth="1"/>
-    <col min="15" max="15" width="17.44140625" customWidth="1"/>
-    <col min="22" max="22" width="17.88671875" customWidth="1"/>
+    <col min="1" max="1" width="15.125" customWidth="1"/>
+    <col min="8" max="8" width="20.125" customWidth="1"/>
+    <col min="15" max="15" width="17.5" customWidth="1"/>
+    <col min="22" max="22" width="17.875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="B1" s="1" t="s">
         <v>6</v>
       </c>
@@ -489,7 +520,7 @@
       <c r="E1" s="1"/>
       <c r="F1" s="1"/>
     </row>
-    <row r="2" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:20" x14ac:dyDescent="0.25">
       <c r="B2" t="s">
         <v>0</v>
       </c>
@@ -506,7 +537,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>5</v>
       </c>
@@ -526,7 +557,7 @@
         <v>0.97060000000000002</v>
       </c>
     </row>
-    <row r="13" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:20" x14ac:dyDescent="0.25">
       <c r="B13" s="1" t="s">
         <v>11</v>
       </c>
@@ -547,7 +578,7 @@
       <c r="S13" s="1"/>
       <c r="T13" s="1"/>
     </row>
-    <row r="14" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:20" x14ac:dyDescent="0.25">
       <c r="B14" t="s">
         <v>0</v>
       </c>
@@ -579,7 +610,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="15" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>8</v>
       </c>
@@ -619,7 +650,7 @@
         <v>19996</v>
       </c>
     </row>
-    <row r="16" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>9</v>
       </c>
@@ -659,7 +690,7 @@
         <v>19599</v>
       </c>
     </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>6</v>
       </c>
@@ -707,7 +738,7 @@
         <v>0.98014602920584115</v>
       </c>
     </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>8</v>
       </c>
@@ -747,7 +778,7 @@
         <v>19996</v>
       </c>
     </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>9</v>
       </c>
@@ -787,7 +818,7 @@
         <v>19673</v>
       </c>
     </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>6</v>
       </c>
@@ -835,7 +866,7 @@
         <v>0.98384676935387072</v>
       </c>
     </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>8</v>
       </c>
@@ -875,7 +906,7 @@
         <v>19996</v>
       </c>
     </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>9</v>
       </c>
@@ -915,7 +946,7 @@
         <v>19504</v>
       </c>
     </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>6</v>
       </c>
@@ -963,7 +994,7 @@
         <v>0.97539507901580313</v>
       </c>
     </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>12</v>
       </c>
@@ -1011,7 +1042,7 @@
         <v>0.97979595919183826</v>
       </c>
     </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:13" x14ac:dyDescent="0.25">
       <c r="B28" s="1" t="s">
         <v>15</v>
       </c>
@@ -1027,7 +1058,7 @@
       <c r="L28" s="1"/>
       <c r="M28" s="1"/>
     </row>
-    <row r="29" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:13" x14ac:dyDescent="0.25">
       <c r="B29" t="s">
         <v>0</v>
       </c>
@@ -1059,7 +1090,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="30" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>8</v>
       </c>
@@ -1099,7 +1130,7 @@
         <v>19998</v>
       </c>
     </row>
-    <row r="31" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>9</v>
       </c>
@@ -1139,7 +1170,7 @@
         <v>19561</v>
       </c>
     </row>
-    <row r="32" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>6</v>
       </c>
@@ -1187,7 +1218,7 @@
         <v>0.97814781478147816</v>
       </c>
     </row>
-    <row r="43" spans="8:13" x14ac:dyDescent="0.3">
+    <row r="43" spans="8:13" x14ac:dyDescent="0.25">
       <c r="I43" s="1" t="s">
         <v>14</v>
       </c>
@@ -1196,7 +1227,7 @@
       <c r="L43" s="1"/>
       <c r="M43" s="1"/>
     </row>
-    <row r="44" spans="8:13" x14ac:dyDescent="0.3">
+    <row r="44" spans="8:13" x14ac:dyDescent="0.25">
       <c r="J44" t="s">
         <v>1</v>
       </c>
@@ -1207,7 +1238,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="45" spans="8:13" x14ac:dyDescent="0.3">
+    <row r="45" spans="8:13" x14ac:dyDescent="0.25">
       <c r="H45" t="s">
         <v>8</v>
       </c>
@@ -1222,7 +1253,7 @@
         <v>19999</v>
       </c>
     </row>
-    <row r="46" spans="8:13" x14ac:dyDescent="0.3">
+    <row r="46" spans="8:13" x14ac:dyDescent="0.25">
       <c r="H46" t="s">
         <v>9</v>
       </c>
@@ -1237,7 +1268,7 @@
         <v>6222</v>
       </c>
     </row>
-    <row r="47" spans="8:13" x14ac:dyDescent="0.3">
+    <row r="47" spans="8:13" x14ac:dyDescent="0.25">
       <c r="H47" t="s">
         <v>6</v>
       </c>
@@ -1254,59 +1285,135 @@
         <v>0.31111555577778888</v>
       </c>
     </row>
-    <row r="58" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:48" x14ac:dyDescent="0.25">
       <c r="B58" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C58" s="1"/>
       <c r="D58" s="1"/>
       <c r="E58" s="1"/>
       <c r="F58" s="1"/>
       <c r="I58" s="1" t="s">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="J58" s="1"/>
       <c r="K58" s="1"/>
       <c r="L58" s="1"/>
       <c r="M58" s="1"/>
       <c r="P58" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="Q58" s="1"/>
       <c r="R58" s="1"/>
       <c r="S58" s="1"/>
       <c r="T58" s="1"/>
-    </row>
-    <row r="59" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="W58" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="X58" s="1"/>
+      <c r="Y58" s="1"/>
+      <c r="Z58" s="1"/>
+      <c r="AA58" s="1"/>
+      <c r="AD58" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="AE58" s="1"/>
+      <c r="AF58" s="1"/>
+      <c r="AG58" s="1"/>
+      <c r="AH58" s="1"/>
+      <c r="AK58" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="AL58" s="1"/>
+      <c r="AM58" s="1"/>
+      <c r="AN58" s="1"/>
+      <c r="AO58" s="1"/>
+      <c r="AR58" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="AS58" s="1"/>
+      <c r="AT58" s="1"/>
+      <c r="AU58" s="1"/>
+      <c r="AV58" s="1"/>
+    </row>
+    <row r="59" spans="1:48" x14ac:dyDescent="0.25">
       <c r="B59" t="s">
-        <v>17</v>
+        <v>16</v>
+      </c>
+      <c r="C59" t="s">
+        <v>22</v>
       </c>
       <c r="F59" t="s">
         <v>7</v>
       </c>
       <c r="I59" t="s">
-        <v>17</v>
+        <v>16</v>
+      </c>
+      <c r="J59" t="s">
+        <v>22</v>
       </c>
       <c r="M59" t="s">
         <v>7</v>
       </c>
       <c r="P59" t="s">
-        <v>17</v>
+        <v>16</v>
+      </c>
+      <c r="Q59" t="s">
+        <v>22</v>
       </c>
       <c r="T59" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="60" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="W59" t="s">
+        <v>16</v>
+      </c>
+      <c r="X59" t="s">
+        <v>22</v>
+      </c>
+      <c r="AA59" t="s">
+        <v>7</v>
+      </c>
+      <c r="AD59" t="s">
+        <v>16</v>
+      </c>
+      <c r="AE59" t="s">
+        <v>22</v>
+      </c>
+      <c r="AH59" t="s">
+        <v>7</v>
+      </c>
+      <c r="AK59" t="s">
+        <v>16</v>
+      </c>
+      <c r="AL59" t="s">
+        <v>22</v>
+      </c>
+      <c r="AO59" t="s">
+        <v>7</v>
+      </c>
+      <c r="AR59" t="s">
+        <v>16</v>
+      </c>
+      <c r="AS59" t="s">
+        <v>22</v>
+      </c>
+      <c r="AV59" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="60" spans="1:48" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>8</v>
       </c>
       <c r="B60">
         <v>10000</v>
       </c>
+      <c r="C60">
+        <v>20000</v>
+      </c>
       <c r="F60">
         <f>SUM(B60:E60)</f>
-        <v>10000</v>
+        <v>30000</v>
       </c>
       <c r="H60" t="s">
         <v>8</v>
@@ -1314,9 +1421,12 @@
       <c r="I60">
         <v>10000</v>
       </c>
+      <c r="J60">
+        <v>20000</v>
+      </c>
       <c r="M60">
         <f>SUM(I60:L60)</f>
-        <v>10000</v>
+        <v>30000</v>
       </c>
       <c r="O60" t="s">
         <v>8</v>
@@ -1324,21 +1434,79 @@
       <c r="P60">
         <v>10000</v>
       </c>
+      <c r="Q60">
+        <v>20000</v>
+      </c>
       <c r="T60">
         <f>SUM(P60:S60)</f>
+        <v>30000</v>
+      </c>
+      <c r="V60" t="s">
+        <v>8</v>
+      </c>
+      <c r="W60">
         <v>10000</v>
       </c>
-    </row>
-    <row r="61" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="X60">
+        <v>20000</v>
+      </c>
+      <c r="AA60">
+        <f>SUM(W60:Z60)</f>
+        <v>30000</v>
+      </c>
+      <c r="AC60" t="s">
+        <v>8</v>
+      </c>
+      <c r="AD60">
+        <v>10000</v>
+      </c>
+      <c r="AE60">
+        <v>20000</v>
+      </c>
+      <c r="AH60">
+        <f>SUM(AD60:AG60)</f>
+        <v>30000</v>
+      </c>
+      <c r="AJ60" t="s">
+        <v>8</v>
+      </c>
+      <c r="AK60">
+        <v>10000</v>
+      </c>
+      <c r="AL60">
+        <v>20000</v>
+      </c>
+      <c r="AO60">
+        <f>SUM(AK60:AN60)</f>
+        <v>30000</v>
+      </c>
+      <c r="AQ60" t="s">
+        <v>8</v>
+      </c>
+      <c r="AR60">
+        <v>10000</v>
+      </c>
+      <c r="AS60">
+        <v>20000</v>
+      </c>
+      <c r="AV60">
+        <f>SUM(AR60:AU60)</f>
+        <v>30000</v>
+      </c>
+    </row>
+    <row r="61" spans="1:48" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>9</v>
       </c>
       <c r="B61">
         <v>6382</v>
       </c>
+      <c r="C61">
+        <v>15282</v>
+      </c>
       <c r="F61">
         <f>SUM(B61:E61)</f>
-        <v>6382</v>
+        <v>21664</v>
       </c>
       <c r="H61" t="s">
         <v>9</v>
@@ -1346,9 +1514,12 @@
       <c r="I61">
         <v>5745</v>
       </c>
+      <c r="J61">
+        <v>16036</v>
+      </c>
       <c r="M61">
         <f>SUM(I61:L61)</f>
-        <v>5745</v>
+        <v>21781</v>
       </c>
       <c r="O61" t="s">
         <v>9</v>
@@ -1356,12 +1527,67 @@
       <c r="P61">
         <v>5744</v>
       </c>
+      <c r="Q61">
+        <v>16067</v>
+      </c>
       <c r="T61">
         <f>SUM(P61:S61)</f>
-        <v>5744</v>
-      </c>
-    </row>
-    <row r="62" spans="1:20" x14ac:dyDescent="0.3">
+        <v>21811</v>
+      </c>
+      <c r="V61" t="s">
+        <v>9</v>
+      </c>
+      <c r="W61">
+        <v>5520</v>
+      </c>
+      <c r="X61">
+        <v>16360</v>
+      </c>
+      <c r="AA61">
+        <f>SUM(W61:Z61)</f>
+        <v>21880</v>
+      </c>
+      <c r="AC61" t="s">
+        <v>9</v>
+      </c>
+      <c r="AD61">
+        <v>5428</v>
+      </c>
+      <c r="AE61">
+        <v>16104</v>
+      </c>
+      <c r="AH61">
+        <f>SUM(AD61:AG61)</f>
+        <v>21532</v>
+      </c>
+      <c r="AJ61" t="s">
+        <v>9</v>
+      </c>
+      <c r="AK61">
+        <v>5379</v>
+      </c>
+      <c r="AL61">
+        <v>16311</v>
+      </c>
+      <c r="AO61">
+        <f>SUM(AK61:AN61)</f>
+        <v>21690</v>
+      </c>
+      <c r="AQ61" t="s">
+        <v>9</v>
+      </c>
+      <c r="AR61">
+        <v>4566</v>
+      </c>
+      <c r="AS61">
+        <v>16111</v>
+      </c>
+      <c r="AV61">
+        <f>SUM(AR61:AU61)</f>
+        <v>20677</v>
+      </c>
+    </row>
+    <row r="62" spans="1:48" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>6</v>
       </c>
@@ -1369,9 +1595,13 @@
         <f t="shared" ref="B62" si="19">B61/B60</f>
         <v>0.63819999999999999</v>
       </c>
+      <c r="C62">
+        <f>C61/C60</f>
+        <v>0.7641</v>
+      </c>
       <c r="F62">
         <f t="shared" ref="F62" si="20">F61/F60</f>
-        <v>0.63819999999999999</v>
+        <v>0.72213333333333329</v>
       </c>
       <c r="H62" t="s">
         <v>6</v>
@@ -1380,9 +1610,13 @@
         <f>I61/I60</f>
         <v>0.57450000000000001</v>
       </c>
+      <c r="J62">
+        <f>J61/J60</f>
+        <v>0.80179999999999996</v>
+      </c>
       <c r="M62">
         <f t="shared" ref="M62" si="21">M61/M60</f>
-        <v>0.57450000000000001</v>
+        <v>0.72603333333333331</v>
       </c>
       <c r="O62" t="s">
         <v>6</v>
@@ -1391,14 +1625,77 @@
         <f t="shared" ref="P62" si="22">P61/P60</f>
         <v>0.57440000000000002</v>
       </c>
+      <c r="Q62">
+        <f>Q61/Q60</f>
+        <v>0.80335000000000001</v>
+      </c>
       <c r="T62">
         <f t="shared" ref="T62" si="23">T61/T60</f>
-        <v>0.57440000000000002</v>
+        <v>0.72703333333333331</v>
+      </c>
+      <c r="V62" t="s">
+        <v>6</v>
+      </c>
+      <c r="W62">
+        <f t="shared" ref="W62" si="24">W61/W60</f>
+        <v>0.55200000000000005</v>
+      </c>
+      <c r="X62">
+        <f>X61/X60</f>
+        <v>0.81799999999999995</v>
+      </c>
+      <c r="AA62">
+        <f t="shared" ref="AA62" si="25">AA61/AA60</f>
+        <v>0.72933333333333328</v>
+      </c>
+      <c r="AC62" t="s">
+        <v>6</v>
+      </c>
+      <c r="AD62">
+        <f t="shared" ref="AD62" si="26">AD61/AD60</f>
+        <v>0.54279999999999995</v>
+      </c>
+      <c r="AE62">
+        <f>AE61/AE60</f>
+        <v>0.80520000000000003</v>
+      </c>
+      <c r="AH62">
+        <f t="shared" ref="AH62" si="27">AH61/AH60</f>
+        <v>0.71773333333333333</v>
+      </c>
+      <c r="AJ62" t="s">
+        <v>6</v>
+      </c>
+      <c r="AK62">
+        <f t="shared" ref="AK62" si="28">AK61/AK60</f>
+        <v>0.53790000000000004</v>
+      </c>
+      <c r="AL62">
+        <f>AL61/AL60</f>
+        <v>0.81555</v>
+      </c>
+      <c r="AO62">
+        <f t="shared" ref="AO62" si="29">AO61/AO60</f>
+        <v>0.72299999999999998</v>
+      </c>
+      <c r="AQ62" t="s">
+        <v>6</v>
+      </c>
+      <c r="AR62">
+        <f t="shared" ref="AR62" si="30">AR61/AR60</f>
+        <v>0.45660000000000001</v>
+      </c>
+      <c r="AS62">
+        <f>AS61/AS60</f>
+        <v>0.80554999999999999</v>
+      </c>
+      <c r="AV62">
+        <f t="shared" ref="AV62" si="31">AV61/AV60</f>
+        <v>0.68923333333333336</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="10">
-    <mergeCell ref="I58:M58"/>
+  <mergeCells count="14">
     <mergeCell ref="P13:T13"/>
     <mergeCell ref="P58:T58"/>
     <mergeCell ref="B58:F58"/>
@@ -1408,6 +1705,11 @@
     <mergeCell ref="I28:M28"/>
     <mergeCell ref="I43:M43"/>
     <mergeCell ref="B28:F28"/>
+    <mergeCell ref="W58:AA58"/>
+    <mergeCell ref="AD58:AH58"/>
+    <mergeCell ref="AR58:AV58"/>
+    <mergeCell ref="AK58:AO58"/>
+    <mergeCell ref="I58:M58"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>